<commit_message>
Re-freeze the metric fixtures for the corrected outlier weight
The only column that moves is weight_outliers, from the quartile fix in
f12383e and its propagation to the synthetic arm in c21f64d:

    TABLE_EmpiricalECCMetrics        weight_outliers      3/149    0.0614 -> 0.0656
                                     weight_outliers_uw   1/149    0.0590 -> 0.0612
    TABLE_EmpiricalECCMetricsAndW1   same
    TABLE_SyntheticECCMetricsAndW1   weight_outliers    474/10000  0.0540 -> 0.0609
                                     weight_outliers_uw 163/10000  0.0526 -> 0.0580

No W1 column moves on either arm. 273 tests pass.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/TABLE_EmpiricalECCMetrics.xlsx
+++ b/tests/fixtures/TABLE_EmpiricalECCMetrics.xlsx
@@ -1751,10 +1751,10 @@
         <v>0.09293681618496408</v>
       </c>
       <c r="V18" t="n">
-        <v>0</v>
+        <v>0.3622193416706191</v>
       </c>
       <c r="W18" t="n">
-        <v>0</v>
+        <v>0.3333333333333333</v>
       </c>
     </row>
     <row r="19">
@@ -4736,7 +4736,7 @@
         <v>0.009230255466642488</v>
       </c>
       <c r="V59" t="n">
-        <v>0</v>
+        <v>0.2482240629063026</v>
       </c>
       <c r="W59" t="n">
         <v>0</v>
@@ -11229,7 +11229,7 @@
         <v>0.2444793042576891</v>
       </c>
       <c r="V148" t="n">
-        <v>0</v>
+        <v>0.01969552426254956</v>
       </c>
       <c r="W148" t="n">
         <v>0.1428571428571428</v>

</xml_diff>